<commit_message>
One new input data set.
</commit_message>
<xml_diff>
--- a/Projects/Example_1_KJ.xlsx
+++ b/Projects/Example_1_KJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KJ\PycharmProjects\MIEcalc3\Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callaghaninnovationgovtnz-my.sharepoint.com/personal/keith_jones_callaghaninnovation_govt_nz/Documents/KJ/PycharmProjects/MIEcalc3/Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2256C0FA-32EC-4BAC-BDC4-0735ED8CCDF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{2256C0FA-32EC-4BAC-BDC4-0735ED8CCDF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF7E4065-4310-478E-9A4F-F0E92E86E011}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="105" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="56175" yWindow="3720" windowWidth="26655" windowHeight="15945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="12" r:id="rId1"/>
@@ -520,7 +520,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -721,6 +721,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -965,7 +971,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -998,6 +1004,8 @@
     <xf numFmtId="164" fontId="0" fillId="34" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="36" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
@@ -11468,29 +11476,27 @@
       <c r="H38" s="25">
         <v>36.918100000000585</v>
       </c>
-      <c r="I38">
-        <v>3.9751834120341688E-2</v>
+      <c r="I38" s="30">
+        <v>0.02</v>
       </c>
       <c r="J38">
         <v>2.1631071081989726</v>
       </c>
-      <c r="K38">
-        <v>1.9271588262657731</v>
+      <c r="K38" s="30">
+        <v>1</v>
       </c>
       <c r="L38" s="14">
         <v>2.2158783911763424</v>
       </c>
-      <c r="N38">
-        <f t="shared" ref="N38:N43" si="0">AVERAGE(C38,E38,G38)</f>
-        <v>-0.2679534192777504</v>
-      </c>
-      <c r="O38">
-        <f t="shared" ref="O38:O43" si="1">RADIANS(AVERAGE(D38,F38,H38)/60)*100</f>
-        <v>1.0587487219627185</v>
-      </c>
-      <c r="P38">
-        <f t="shared" ref="P38:P43" si="2">RADIANS(K38/60)*100</f>
-        <v>5.6058777878678523E-2</v>
+      <c r="N38" s="30">
+        <v>-0.14304438683682899</v>
+      </c>
+      <c r="O38" s="30">
+        <v>0.24077326659739401</v>
+      </c>
+      <c r="P38" s="30">
+        <f t="shared" ref="P38:P43" si="0">RADIANS(K38/60)*100</f>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
@@ -11515,29 +11521,27 @@
       <c r="H39" s="25">
         <v>28.585500000000664</v>
       </c>
-      <c r="I39">
-        <v>3.9746598897763628E-2</v>
+      <c r="I39" s="30">
+        <v>0.02</v>
       </c>
       <c r="J39">
         <v>2.1633007328489464</v>
       </c>
-      <c r="K39">
-        <v>1.9268256542944926</v>
+      <c r="K39" s="30">
+        <v>1</v>
       </c>
       <c r="L39" s="14">
         <v>2.2162774837041446</v>
       </c>
-      <c r="N39">
+      <c r="N39" s="30">
+        <v>-0.12153114192209101</v>
+      </c>
+      <c r="O39" s="30">
+        <v>0.20632604900513402</v>
+      </c>
+      <c r="P39" s="30">
         <f t="shared" si="0"/>
-        <v>-0.15298399182566602</v>
-      </c>
-      <c r="O39">
-        <f t="shared" si="1"/>
-        <v>0.83214680741212022</v>
-      </c>
-      <c r="P39">
-        <f t="shared" si="2"/>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
@@ -11562,29 +11566,27 @@
       <c r="H40" s="25">
         <v>23.222000000000449</v>
       </c>
-      <c r="I40">
-        <v>3.9745633167544044E-2</v>
+      <c r="I40" s="30">
+        <v>0.02</v>
       </c>
       <c r="J40">
         <v>2.1633007328489464</v>
       </c>
-      <c r="K40">
-        <v>1.9268256542944926</v>
+      <c r="K40" s="30">
+        <v>1</v>
       </c>
       <c r="L40" s="14">
         <v>2.2162774837041446</v>
       </c>
-      <c r="N40">
+      <c r="N40" s="30">
+        <v>-0.110920649790078</v>
+      </c>
+      <c r="O40" s="30">
+        <v>0.17721835461164101</v>
+      </c>
+      <c r="P40" s="30">
         <f t="shared" si="0"/>
-        <v>-6.4064893407896312E-2</v>
-      </c>
-      <c r="O40">
-        <f t="shared" si="1"/>
-        <v>0.69748011121031916</v>
-      </c>
-      <c r="P40">
-        <f t="shared" si="2"/>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
@@ -11609,29 +11611,27 @@
       <c r="H41" s="25">
         <v>16.180700000000034</v>
       </c>
-      <c r="I41">
-        <v>3.9745879805498992E-2</v>
+      <c r="I41" s="30">
+        <v>0.02</v>
       </c>
       <c r="J41">
         <v>2.1633007328489464</v>
       </c>
-      <c r="K41">
-        <v>1.9268256542944926</v>
+      <c r="K41" s="30">
+        <v>1</v>
       </c>
       <c r="L41" s="14">
         <v>2.2162774837041446</v>
       </c>
-      <c r="N41">
+      <c r="N41" s="30">
+        <v>-0.10283111238602501</v>
+      </c>
+      <c r="O41" s="30">
+        <v>0.13463441485188901</v>
+      </c>
+      <c r="P41" s="30">
         <f t="shared" si="0"/>
-        <v>4.2024122754677269E-2</v>
-      </c>
-      <c r="O41">
-        <f t="shared" si="1"/>
-        <v>0.52069862015790302</v>
-      </c>
-      <c r="P41">
-        <f t="shared" si="2"/>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
@@ -11656,29 +11656,27 @@
       <c r="H42" s="25">
         <v>15.009600000000724</v>
       </c>
-      <c r="I42">
-        <v>3.9747232821419044E-2</v>
+      <c r="I42" s="30">
+        <v>0.02</v>
       </c>
       <c r="J42">
         <v>2.1633007328489464</v>
       </c>
-      <c r="K42">
-        <v>1.9268256542944926</v>
+      <c r="K42" s="30">
+        <v>1</v>
       </c>
       <c r="L42" s="14">
         <v>2.2162774837041446</v>
       </c>
-      <c r="N42">
+      <c r="N42" s="30">
+        <v>-9.6999508246314106E-2</v>
+      </c>
+      <c r="O42" s="30">
+        <v>0.114612087149039</v>
+      </c>
+      <c r="P42" s="30">
         <f t="shared" si="0"/>
-        <v>7.4202892966420408E-2</v>
-      </c>
-      <c r="O42">
-        <f t="shared" si="1"/>
-        <v>0.43863032984705186</v>
-      </c>
-      <c r="P42">
-        <f t="shared" si="2"/>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
@@ -11703,29 +11701,27 @@
       <c r="H43" s="28">
         <v>15.25330000000003</v>
       </c>
-      <c r="I43" s="19">
-        <v>3.9746659607446784E-2</v>
+      <c r="I43" s="31">
+        <v>0.02</v>
       </c>
       <c r="J43" s="19">
         <v>2.1633007328489464</v>
       </c>
-      <c r="K43" s="19">
-        <v>1.9268256542944926</v>
+      <c r="K43" s="31">
+        <v>1</v>
       </c>
       <c r="L43" s="20">
         <v>2.2162774837041446</v>
       </c>
-      <c r="N43">
+      <c r="N43" s="30">
+        <v>-9.4079004216734208E-2</v>
+      </c>
+      <c r="O43" s="30">
+        <v>0.10755913449750701</v>
+      </c>
+      <c r="P43" s="30">
         <f t="shared" si="0"/>
-        <v>8.0902195356431048E-2</v>
-      </c>
-      <c r="O43">
-        <f t="shared" si="1"/>
-        <v>0.43677737195783684</v>
-      </c>
-      <c r="P43">
-        <f t="shared" si="2"/>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -12634,11 +12630,11 @@
       </c>
       <c r="B3">
         <f>InputData!N38</f>
-        <v>-0.2679534192777504</v>
+        <v>-0.14304438683682899</v>
       </c>
       <c r="C3">
         <f>InputData!I38</f>
-        <v>3.9751834120341688E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D3">
         <f>InputData!J38</f>
@@ -12646,11 +12642,11 @@
       </c>
       <c r="E3">
         <f>InputData!O38</f>
-        <v>1.0587487219627185</v>
+        <v>0.24077326659739401</v>
       </c>
       <c r="F3">
         <f>InputData!P38</f>
-        <v>5.6058777878678523E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G3">
         <f>InputData!L38</f>
@@ -12664,11 +12660,11 @@
       </c>
       <c r="B4">
         <f>InputData!N39</f>
-        <v>-0.15298399182566602</v>
+        <v>-0.12153114192209101</v>
       </c>
       <c r="C4">
         <f>InputData!I39</f>
-        <v>3.9746598897763628E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D4">
         <f>InputData!J39</f>
@@ -12676,11 +12672,11 @@
       </c>
       <c r="E4">
         <f>InputData!O39</f>
-        <v>0.83214680741212022</v>
+        <v>0.20632604900513402</v>
       </c>
       <c r="F4">
         <f>InputData!P39</f>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G4">
         <f>InputData!L39</f>
@@ -12694,11 +12690,11 @@
       </c>
       <c r="B5">
         <f>InputData!N40</f>
-        <v>-6.4064893407896312E-2</v>
+        <v>-0.110920649790078</v>
       </c>
       <c r="C5">
         <f>InputData!I40</f>
-        <v>3.9745633167544044E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D5">
         <f>InputData!J40</f>
@@ -12706,11 +12702,11 @@
       </c>
       <c r="E5">
         <f>InputData!O40</f>
-        <v>0.69748011121031916</v>
+        <v>0.17721835461164101</v>
       </c>
       <c r="F5">
         <f>InputData!P40</f>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G5">
         <f>InputData!L40</f>
@@ -12724,11 +12720,11 @@
       </c>
       <c r="B6">
         <f>InputData!N41</f>
-        <v>4.2024122754677269E-2</v>
+        <v>-0.10283111238602501</v>
       </c>
       <c r="C6">
         <f>InputData!I41</f>
-        <v>3.9745879805498992E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D6">
         <f>InputData!J41</f>
@@ -12736,11 +12732,11 @@
       </c>
       <c r="E6">
         <f>InputData!O41</f>
-        <v>0.52069862015790302</v>
+        <v>0.13463441485188901</v>
       </c>
       <c r="F6">
         <f>InputData!P41</f>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G6">
         <f>InputData!L41</f>
@@ -12754,11 +12750,11 @@
       </c>
       <c r="B7">
         <f>InputData!N42</f>
-        <v>7.4202892966420408E-2</v>
+        <v>-9.6999508246314106E-2</v>
       </c>
       <c r="C7">
         <f>InputData!I42</f>
-        <v>3.9747232821419044E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D7">
         <f>InputData!J42</f>
@@ -12766,11 +12762,11 @@
       </c>
       <c r="E7">
         <f>InputData!O42</f>
-        <v>0.43863032984705186</v>
+        <v>0.114612087149039</v>
       </c>
       <c r="F7">
         <f>InputData!P42</f>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G7">
         <f>InputData!L42</f>
@@ -12784,11 +12780,11 @@
       </c>
       <c r="B8">
         <f>InputData!N43</f>
-        <v>8.0902195356431048E-2</v>
+        <v>-9.4079004216734208E-2</v>
       </c>
       <c r="C8">
         <f>InputData!I43</f>
-        <v>3.9746659607446784E-2</v>
+        <v>0.02</v>
       </c>
       <c r="D8">
         <f>InputData!J43</f>
@@ -12796,11 +12792,11 @@
       </c>
       <c r="E8">
         <f>InputData!O43</f>
-        <v>0.43677737195783684</v>
+        <v>0.10755913449750701</v>
       </c>
       <c r="F8">
         <f>InputData!P43</f>
-        <v>5.604908629888819E-2</v>
+        <v>2.9088820866572159E-2</v>
       </c>
       <c r="G8">
         <f>InputData!L43</f>

</xml_diff>